<commit_message>
el code 128 de la hoja de codigos extra ya no sobresale de la etiqueta
El Code 128 mide casi lo mismo que el ancho util de la etiqueta (2.118.833
EMU frente a 2.161.629 de las columnas 6 y 7), asi que con el dx anterior
(60959) el borde derecho caia ~18.000 EMU fuera. Se corre ~3 pt a la
izquierda, igual que en la plantilla de referencia del cliente.

El tamano NO se toca: reescalar un codigo de barras lo deja bonito en
pantalla e ilegible para un lector fisico.

El anclaje de las imagenes no lo miraba ningun test; ahora la maquetacion
lo compara con la plantilla, con 1 pixel de tolerancia porque alli las tres
copias estan puestas a mano y no coinciden entre si.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Etiquetas cajas/AMI ETIQUETAS CAJA - CODE BARRAS EXTRA TEMPLATE.xlsx
+++ b/docs/Etiquetas cajas/AMI ETIQUETAS CAJA - CODE BARRAS EXTRA TEMPLATE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jordi\Documents\Workspace\Packing List Automation\docs\Etiquetas cajas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CC54ED3F-A360-4551-903A-95C1FB2A6473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B113B613-C999-4564-98ED-975ECB52D152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{02BB6957-E6F7-49EE-B2B6-A2C9861D9CAC}"/>
   </bookViews>
@@ -147,13 +147,13 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -228,13 +228,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>60959</xdr:colOff>
+      <xdr:colOff>22859</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>144780</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>1173952</xdr:colOff>
+      <xdr:colOff>1135852</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>131259</xdr:rowOff>
     </xdr:to>
@@ -266,7 +266,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="4777739" y="586740"/>
+          <a:off x="4739639" y="586740"/>
           <a:ext cx="2118833" cy="352239"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -334,13 +334,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>68580</xdr:colOff>
+      <xdr:colOff>22860</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>129540</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>1181573</xdr:colOff>
+      <xdr:colOff>1135853</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>116019</xdr:rowOff>
     </xdr:to>
@@ -372,7 +372,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="4785360" y="1973580"/>
+          <a:off x="4739640" y="1973580"/>
           <a:ext cx="2118833" cy="352239"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -440,7 +440,7 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>53340</xdr:colOff>
+      <xdr:colOff>30480</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>129540</xdr:rowOff>
     </xdr:from>
@@ -473,7 +473,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="4770120" y="3375660"/>
+          <a:off x="4747260" y="3375660"/>
           <a:ext cx="2118833" cy="352239"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -811,10 +811,10 @@
   <sheetData>
     <row r="1" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>5</v>
       </c>
       <c r="C2" s="1"/>
@@ -834,8 +834,8 @@
       <c r="K2" s="1"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="4"/>
-      <c r="B3" s="5"/>
+      <c r="A3" s="5"/>
+      <c r="B3" s="6"/>
       <c r="C3" s="1"/>
       <c r="D3" s="3" t="s">
         <v>2</v>
@@ -854,23 +854,23 @@
       <c r="K3" s="1"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6"/>
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
     </row>
     <row r="9" spans="1:11" ht="9.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D10" t="s">
@@ -887,8 +887,8 @@
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="4"/>
-      <c r="B11" s="5"/>
+      <c r="A11" s="5"/>
+      <c r="B11" s="6"/>
       <c r="D11" s="3" t="s">
         <v>2</v>
       </c>
@@ -903,23 +903,23 @@
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="6"/>
-      <c r="B13" s="6"/>
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
     </row>
     <row r="17" spans="1:8" ht="9.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="6" t="s">
         <v>9</v>
       </c>
       <c r="D18" t="s">
@@ -936,8 +936,8 @@
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="4"/>
-      <c r="B19" s="5"/>
+      <c r="A19" s="5"/>
+      <c r="B19" s="6"/>
       <c r="D19" s="3" t="s">
         <v>2</v>
       </c>
@@ -952,16 +952,16 @@
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" s="6"/>
-      <c r="B21" s="6"/>
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
     </row>
     <row r="25" spans="1:8" ht="9.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -973,18 +973,18 @@
     <row r="73" ht="9.9" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B10:B11"/>
     <mergeCell ref="A12:A13"/>
     <mergeCell ref="B12:B13"/>
     <mergeCell ref="A18:A19"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="A20:A21"/>
     <mergeCell ref="B20:B21"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="B10:B11"/>
   </mergeCells>
   <pageMargins left="0" right="3.937007874015748E-2" top="3.937007874015748E-2" bottom="3.937007874015748E-2" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="74" orientation="portrait" r:id="rId1"/>

</xml_diff>